<commit_message>
made changes to the user interface and added functionality
</commit_message>
<xml_diff>
--- a/sample_data/programme_courses.xlsx
+++ b/sample_data/programme_courses.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,16 @@
           <t>course_code</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>course_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>semester</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +449,14 @@
           <t>MT161</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mathematics 1</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +469,14 @@
           <t>TG201</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Technical Drawing 1</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,6 +489,14 @@
           <t>ST101</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Statistics 1</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -475,6 +509,14 @@
           <t>MT161</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mathematics 1</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -487,6 +529,14 @@
           <t>EE101</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Electrical Engineering 1</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -499,6 +549,14 @@
           <t>MT161</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mathematics 1</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -511,6 +569,14 @@
           <t>ME101</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mechanical Engineering 1</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -522,6 +588,14 @@
         <is>
           <t>IE101</t>
         </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Industrial Engineering 1</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>